<commit_message>
Renderizando el libro para GitHub Pages
</commit_message>
<xml_diff>
--- a/FORMULARIO/CRONO.xlsx
+++ b/FORMULARIO/CRONO.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
   <si>
     <t xml:space="preserve">N</t>
   </si>
@@ -515,6 +515,12 @@
       </rPr>
       <t xml:space="preserve">(ASPLENIACEAE) DE LAS YUNGAS ARGENTINAS, MEDIANTE LA APLICACION DE TECNICAS DE LABORATORIO CONVENCIONALES.</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ESTUDIO DE PARÁMETROS REPRODUCTIVOS EN OVINOS CON VISTAS AL MEJORAMIENTO GENÉTICO EN LA ECOREGIÓN PUNA. PROVINCIA DE JUJUY </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAPA DE FERTILIDAD CON USO DE VARIABLES FÍSICAS-QUÍMICAS DEL SUELO DEL CAMPO EXPERIMENTAL DR. EMILIO NAVEA, FCA-UNJu </t>
   </si>
 </sst>
 </file>
@@ -524,7 +530,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -561,6 +567,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri-BoldItalic"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -622,7 +636,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -634,8 +648,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -647,31 +661,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF6D"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -915,13 +904,13 @@
   <dimension ref="A1:C1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="91.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="91.98"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1158,7 +1147,7 @@
       <c r="B22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="3" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1169,7 +1158,7 @@
       <c r="B23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="3" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1180,7 +1169,7 @@
       <c r="B24" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="3" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1191,7 +1180,7 @@
       <c r="B25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1202,7 +1191,7 @@
       <c r="B26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="3" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1213,7 +1202,7 @@
       <c r="B27" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="3" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1224,7 +1213,7 @@
       <c r="B28" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1235,7 +1224,7 @@
       <c r="B29" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="3" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1246,7 +1235,7 @@
       <c r="B30" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="3" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1257,8 +1246,30 @@
       <c r="B31" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="3" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>